<commit_message>
analysis: first chart — category speedups (membound146, bw3200) + ledger updates
</commit_message>
<xml_diff>
--- a/analysis/hermes_results.xlsx
+++ b/analysis/hermes_results.xlsx
@@ -476,7 +476,11 @@
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>speedup_membound146_bw3200.{png,pdf}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -658,9 +662,6 @@
       <c r="C7" t="n">
         <v>1.8735</v>
       </c>
-      <c r="D7" t="n">
-        <v/>
-      </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -778,9 +779,6 @@
       <c r="C12" t="n">
         <v>0.45542</v>
       </c>
-      <c r="D12" t="n">
-        <v/>
-      </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
@@ -802,9 +800,6 @@
       <c r="C13" t="n">
         <v>0.53765</v>
       </c>
-      <c r="D13" t="n">
-        <v/>
-      </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
@@ -1090,9 +1085,6 @@
       <c r="C25" t="n">
         <v>1.08084</v>
       </c>
-      <c r="D25" t="n">
-        <v/>
-      </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
@@ -3970,9 +3962,6 @@
       <c r="C145" t="n">
         <v>1.20226</v>
       </c>
-      <c r="D145" t="n">
-        <v/>
-      </c>
       <c r="E145" t="n">
         <v>0</v>
       </c>
@@ -5554,9 +5543,6 @@
       <c r="C211" t="n">
         <v>0.64459</v>
       </c>
-      <c r="D211" t="n">
-        <v/>
-      </c>
       <c r="E211" t="n">
         <v>0</v>
       </c>
@@ -9586,9 +9572,6 @@
       <c r="C379" t="n">
         <v>0.73336</v>
       </c>
-      <c r="D379" t="n">
-        <v/>
-      </c>
       <c r="E379" t="n">
         <v>0</v>
       </c>
@@ -9874,9 +9857,6 @@
       <c r="C391" t="n">
         <v>0.73286</v>
       </c>
-      <c r="D391" t="n">
-        <v/>
-      </c>
       <c r="E391" t="n">
         <v>0</v>
       </c>
@@ -10738,9 +10718,6 @@
       <c r="C427" t="n">
         <v>1.27634</v>
       </c>
-      <c r="D427" t="n">
-        <v/>
-      </c>
       <c r="E427" t="n">
         <v>0</v>
       </c>
@@ -10882,9 +10859,6 @@
       <c r="C433" t="n">
         <v>2.06589</v>
       </c>
-      <c r="D433" t="n">
-        <v/>
-      </c>
       <c r="E433" t="n">
         <v>0</v>
       </c>
@@ -11026,9 +11000,6 @@
       <c r="C439" t="n">
         <v>1.99553</v>
       </c>
-      <c r="D439" t="n">
-        <v/>
-      </c>
       <c r="E439" t="n">
         <v>0</v>
       </c>
@@ -17650,9 +17621,6 @@
       <c r="C715" t="n">
         <v>1.56396</v>
       </c>
-      <c r="D715" t="n">
-        <v/>
-      </c>
       <c r="E715" t="n">
         <v>0</v>
       </c>
@@ -18082,9 +18050,6 @@
       <c r="C733" t="n">
         <v>0.81303</v>
       </c>
-      <c r="D733" t="n">
-        <v/>
-      </c>
       <c r="E733" t="n">
         <v>0</v>
       </c>
@@ -19522,9 +19487,6 @@
       <c r="C793" t="n">
         <v>0.96675</v>
       </c>
-      <c r="D793" t="n">
-        <v/>
-      </c>
       <c r="E793" t="n">
         <v>0</v>
       </c>
@@ -19810,9 +19772,6 @@
       <c r="C805" t="n">
         <v>0.97387</v>
       </c>
-      <c r="D805" t="n">
-        <v/>
-      </c>
       <c r="E805" t="n">
         <v>0</v>
       </c>
@@ -20386,9 +20345,6 @@
       <c r="C829" t="n">
         <v>0.5414</v>
       </c>
-      <c r="D829" t="n">
-        <v/>
-      </c>
       <c r="E829" t="n">
         <v>0</v>
       </c>
@@ -21393,9 +21349,6 @@
       </c>
       <c r="C871" t="n">
         <v>0.95261</v>
-      </c>
-      <c r="D871" t="n">
-        <v/>
       </c>
       <c r="E871" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
analysis: accuracy/coverage chart (XPT vs Hermes-UnC) + excel sheet + index
</commit_message>
<xml_diff>
--- a/analysis/hermes_results.xlsx
+++ b/analysis/hermes_results.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDEX" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="membound146_bw3200" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="accuracy_coverage_bw3200" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -478,7 +479,34 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>speedup_membound146_bw3200.{png,pdf}</t>
+          <t>speedup_membound146_bw3200; accuracy_coverage_membound146_bw3200 (raw precision/recall live in this sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>accuracy_coverage_bw3200</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Per-category AVG accuracy(precision)/coverage(recall), XPT &amp; Hermes-UnC standalone (non-weighted arith mean; XPT accuracy n=145, 1 zero-prediction trace excluded)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>derived from membound146_bw3200</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>accuracy_coverage_membound146_bw3200</t>
         </is>
       </c>
     </row>
@@ -21504,4 +21532,512 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ExpName</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>95.517397260274</v>
+      </c>
+      <c r="E2" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>97.6444827586207</v>
+      </c>
+      <c r="E3" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>96.72133333333331</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>98.6816666666667</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>95.8235714285714</v>
+      </c>
+      <c r="E6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>98.8644444444444</v>
+      </c>
+      <c r="E7" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>99.1953125</v>
+      </c>
+      <c r="E8" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>95.8184375</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>92.6176785714286</v>
+      </c>
+      <c r="E10" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>97.5441071428571</v>
+      </c>
+      <c r="E11" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>94.9815753424658</v>
+      </c>
+      <c r="E12" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>25.5078082191781</v>
+      </c>
+      <c r="E13" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>97.4146666666667</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>31.4856666666667</v>
+      </c>
+      <c r="E15" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>96.1278571428571</v>
+      </c>
+      <c r="E16" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>19.0228571428571</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>97.109375</v>
+      </c>
+      <c r="E18" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>39.298125</v>
+      </c>
+      <c r="E19" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Hermes-UnC</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>91.8891071428571</v>
+      </c>
+      <c r="E20" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>XPT</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>17.6676785714286</v>
+      </c>
+      <c r="E21" t="n">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
analysis: accuracy/coverage +Pythia variant + benefit-of-doubt rule; two variant sheets
</commit_message>
<xml_diff>
--- a/analysis/hermes_results.xlsx
+++ b/analysis/hermes_results.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDEX" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="membound146_bw3200" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="accuracy_coverage_bw3200" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="acc_cov_standalone_bw3200" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="acc_cov_pythia_bw3200" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -479,34 +480,62 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>speedup_membound146_bw3200; accuracy_coverage_membound146_bw3200 (raw precision/recall live in this sheet)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>accuracy_coverage_bw3200</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Per-category AVG accuracy(precision)/coverage(recall), XPT &amp; Hermes-UnC standalone (non-weighted arith mean; XPT accuracy n=145, 1 zero-prediction trace excluded)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>speedup_membound146_bw3200; accuracy_coverage_{standalone,pythia}_membound146_bw3200 (raw precision/recall live here)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>acc_cov_standalone_bw3200</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Per-cat AVG accuracy/coverage, XPT &amp; Hermes-UnC standalone (arith mean; no-prediction=100% accuracy)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>derived from membound146_bw3200</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>accuracy_coverage_membound146_bw3200</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>accuracy_coverage_standalone_membound146_bw3200</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>acc_cov_pythia_bw3200</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Per-cat AVG accuracy/coverage, XPT+Pythia &amp; Hermes-UnC+Pythia (arith mean; no-prediction=100% accuracy; 16 XPT no-pred traces)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>derived from membound146_bw3200</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>accuracy_coverage_pythia_membound146_bw3200</t>
         </is>
       </c>
     </row>
@@ -21545,7 +21574,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -21617,10 +21646,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>97.6444827586207</v>
+        <v>97.6606164383562</v>
       </c>
       <c r="E3" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4">
@@ -21709,10 +21738,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>98.8644444444444</v>
+        <v>98.905</v>
       </c>
       <c r="E7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -22032,6 +22061,514 @@
       </c>
       <c r="D21" t="n">
         <v>17.6676785714286</v>
+      </c>
+      <c r="E21" t="n">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ExpName</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>85.4189726027397</v>
+      </c>
+      <c r="E2" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>65.386095890411</v>
+      </c>
+      <c r="E3" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>88.01066666666669</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>69.3606666666667</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>88.27035714285709</v>
+      </c>
+      <c r="E6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>67.85892857142861</v>
+      </c>
+      <c r="E7" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>87.8384375</v>
+      </c>
+      <c r="E8" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>71.31874999999999</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>81.22232142857141</v>
+      </c>
+      <c r="E10" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>58.6303571428571</v>
+      </c>
+      <c r="E11" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>69.84321917808219</v>
+      </c>
+      <c r="E12" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5.3877397260274</v>
+      </c>
+      <c r="E13" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>77.51900000000001</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>specrate-fp</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>11.2813333333333</v>
+      </c>
+      <c r="E15" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>75.4089285714286</v>
+      </c>
+      <c r="E16" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>specrate-int</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2.19464285714286</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>62.5840625</v>
+      </c>
+      <c r="E18" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>specspeed-fp</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="E19" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Hermes-UnC+Pythia</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>67.0964285714286</v>
+      </c>
+      <c r="E20" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>specspeed-int</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>XPT+Pythia</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.16857142857143</v>
       </c>
       <c r="E21" t="n">
         <v>56</v>

</xml_diff>